<commit_message>
User checkpoint: Add XLSX output and generate PDF for 152.00_101 HART LANE, LLC.
</commit_message>
<xml_diff>
--- a/outputs/default/output.xlsx
+++ b/outputs/default/output.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,6 +491,68 @@
         <is>
           <t>Tax</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>101 Hart ln</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>101 HART LANE, LLC</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>101 HART LN</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>06012015200</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>152.00</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>664400</v>
+      </c>
+      <c r="I2" t="n">
+        <v>93300</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>40.0%</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>3.254</v>
+      </c>
+      <c r="M2">
+        <f>H2+I2+j2</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>M2*(K2)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>N2*(L2/100)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
User checkpoint: Update output.xlsx.
</commit_message>
<xml_diff>
--- a/outputs/default/output.xlsx
+++ b/outputs/default/output.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,68 +491,6 @@
         <is>
           <t>Tax</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>101 Hart ln</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>101 HART LANE, LLC</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>101 HART LN</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>06012015200</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>152.00</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>664400</v>
-      </c>
-      <c r="I2" t="n">
-        <v>93300</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
-        <v>3.254</v>
-      </c>
-      <c r="M2">
-        <f>H2+I2+j2</f>
-        <v/>
-      </c>
-      <c r="N2">
-        <f>M2*(K2)</f>
-        <v/>
-      </c>
-      <c r="O2">
-        <f>N2*(L2/100)</f>
-        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>